<commit_message>
docs: add framework and design slide assets
Add framework image updates and design slide assets for Video Analyze, Fanarts, and Recreated Page.
</commit_message>
<xml_diff>
--- a/docs/design.xlsx
+++ b/docs/design.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\D\git\Himari-profile\vite-vtb-himari-profile\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F851966-B9C6-4895-A0BE-79B3537B9870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F3DAACE-D247-4C34-8EC1-6ABCA83BD41C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{02134FC4-5CC4-44BC-A41F-4C90AC147F71}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{02134FC4-5CC4-44BC-A41F-4C90AC147F71}"/>
   </bookViews>
   <sheets>
     <sheet name="framework" sheetId="1" r:id="rId1"/>
+    <sheet name="completed-framework" sheetId="4" r:id="rId2"/>
+    <sheet name="completed-block" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -700,6 +702,662 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>251455</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>141442</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="圖片 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B278FAC-4A99-4CF9-A86E-6B8F073E1E20}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="554182" y="831273"/>
+          <a:ext cx="8010000" cy="4505624"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>249493</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>6218</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="圖片 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A597814D-3F95-4E55-9387-6F9EAB67C6B1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="6958" t="8239" r="6958" b="8239"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="554182" y="5611091"/>
+          <a:ext cx="8008038" cy="4370400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>251455</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>92221</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="圖片 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4CC56B57-49E4-4144-9388-C4D0B5384A37}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="5704" t="26619" r="5704" b="26619"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="554182" y="16209818"/>
+          <a:ext cx="8010000" cy="2378221"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>251455</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>69988</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="圖片 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CDDA4537-7FB8-4713-83A8-CF8C444EF25D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect t="21549" b="21549"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="554182" y="13508182"/>
+          <a:ext cx="8010000" cy="2563806"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>251455</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="14" name="矩形 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A6053CBB-EEA4-41FF-AAD9-E66FBDC37798}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="554182" y="10183091"/>
+          <a:ext cx="8010000" cy="3061854"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-TW" sz="5400"/>
+            <a:t>None</a:t>
+          </a:r>
+          <a:endParaRPr lang="zh-TW" altLang="en-US" sz="5400"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3626121" cy="268920"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="20" name="Text Box 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{179B4F63-06BB-4BB1-BDB2-1CDA2A78D76A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1">
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="271670" y="616226"/>
+          <a:ext cx="3626121" cy="268920"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" wrap="none" lIns="27432" tIns="18288" rIns="0" bIns="0" anchor="t" upright="1">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l" rtl="0">
+            <a:defRPr sz="1000"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="zh-TW" altLang="en-US" sz="1600" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="新細明體"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>docs\01-profile\profile-section-design.pptx</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>79755</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>63512</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="21" name="Text Box 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F67E8417-CBF8-426E-8D5A-53745769D072}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1">
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="271670" y="16432696"/>
+          <a:ext cx="4426468" cy="268920"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" wrap="none" lIns="27432" tIns="18288" rIns="0" bIns="0" anchor="t" upright="1">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" indent="0" algn="l" rtl="0">
+            <a:defRPr sz="1000"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="zh-TW" altLang="en-US" sz="1600" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="新細明體"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>docs\05-recreated-page\recreated-page-design.pptx</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>56315</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>63511</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="22" name="Text Box 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{29B0C4BE-A21D-443D-BD5A-74EE2B270308}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1">
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="271670" y="13556974"/>
+          <a:ext cx="3044680" cy="268920"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" wrap="none" lIns="27432" tIns="18288" rIns="0" bIns="0" anchor="t" upright="1">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" indent="0" algn="l" rtl="0">
+            <a:defRPr sz="1000"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="zh-TW" altLang="en-US" sz="1600" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="新細明體"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>docs\04-fanarts\fanarts-design.pptx</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>90585</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>63512</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="23" name="Text Box 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{81088F8E-20BB-4FB1-9CFD-7A77B5E9A2F7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1">
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="271670" y="5546035"/>
+          <a:ext cx="4165628" cy="268920"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" wrap="none" lIns="27432" tIns="18288" rIns="0" bIns="0" anchor="t" upright="1">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" indent="0" algn="l" rtl="0">
+            <a:defRPr sz="1000"/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="zh-TW" altLang="en-US" sz="1600" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="新細明體"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>docs\02-video-analyze\video-analyze-design.pptx</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>251455</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>152399</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="圖片 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C4C94C6-F5EE-494F-96C4-E9A48C055489}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:srcRect b="31195"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="554182" y="831273"/>
+          <a:ext cx="8010000" cy="5347853"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>251455</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>152399</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="圖片 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{077A9E2B-EBE9-4C9D-8863-E32035BB3D65}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:srcRect t="18003" b="31907"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="554182" y="8936182"/>
+          <a:ext cx="8010000" cy="3893126"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 佈景主題">
   <a:themeElements>
@@ -2269,4 +2927,28 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3E41E55-A8DE-4B8A-977C-326B1F4D844D}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="4" defaultRowHeight="16.2"/>
+  <sheetData/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97E09F4F-F0B3-49BE-9C03-968F9A201DA9}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="4" defaultRowHeight="16.2"/>
+  <sheetData/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>